<commit_message>
fix: correct workbook recalculation controls
</commit_message>
<xml_diff>
--- a/frontend/public/template-files/bank-reconciliation-workpaper-template.xlsx
+++ b/frontend/public/template-files/bank-reconciliation-workpaper-template.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="88">
   <si>
     <t>Bank Reconciliation Workpaper</t>
   </si>
@@ -33,7 +33,7 @@
     <t>Bank Account</t>
   </si>
   <si>
-    <t>Operating Account ••4821</t>
+    <t>Operating Account 4821</t>
   </si>
   <si>
     <t>Statement Date</t>
@@ -51,7 +51,7 @@
     <t>Paste Import</t>
   </si>
   <si>
-    <t>Review Date</t>
+    <t>Completion Date</t>
   </si>
   <si>
     <t>Currency</t>
@@ -102,7 +102,7 @@
     <t>Review item or failed control</t>
   </si>
   <si>
-    <t>Paste Import — Bank Reconciliation</t>
+    <t>Paste Import - Bank Reconciliation</t>
   </si>
   <si>
     <t>Statement Balance</t>
@@ -213,16 +213,16 @@
     <t>CLR-0021</t>
   </si>
   <si>
-    <t>Cleared transfer — bank</t>
+    <t>Cleared transfer - bank</t>
   </si>
   <si>
     <t>Matched item</t>
   </si>
   <si>
-    <t>Cleared transfer — books</t>
-  </si>
-  <si>
-    <t>Manual Input — Bank Reconciliation</t>
+    <t>Cleared transfer - books</t>
+  </si>
+  <si>
+    <t>Manual Input - Bank Reconciliation</t>
   </si>
   <si>
     <t>Bank Reconciliation Review</t>
@@ -237,7 +237,7 @@
     <t>Input Check</t>
   </si>
   <si>
-    <t>Bank Reconciliation — Summary</t>
+    <t>Bank Reconciliation - Summary</t>
   </si>
   <si>
     <t>Printable reconciliation control and sign-off workpaper</t>
@@ -3893,7 +3893,7 @@
       </c>
       <c r="C11" s="18" t="str">
         <f>IF('Start Here'!$B$8="Paste Import",'Paste Import'!C11,'Manual Input'!C11)</f>
-        <v>Cleared transfer — bank</v>
+        <v>Cleared transfer - bank</v>
       </c>
       <c r="D11" s="19">
         <f>IF('Start Here'!$B$8="Paste Import",'Paste Import'!D11,'Manual Input'!D11)</f>
@@ -3935,7 +3935,7 @@
       </c>
       <c r="C12" s="18" t="str">
         <f>IF('Start Here'!$B$8="Paste Import",'Paste Import'!C12,'Manual Input'!C12)</f>
-        <v>Cleared transfer — books</v>
+        <v>Cleared transfer - books</v>
       </c>
       <c r="D12" s="19">
         <f>IF('Start Here'!$B$8="Paste Import",'Paste Import'!D12,'Manual Input'!D12)</f>
@@ -7979,7 +7979,15 @@
         <v>Review</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="23" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="24">
+        <f>'Start Here'!B9</f>
+        <v>46213</v>
+      </c>
+    </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25"/>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="26" t="s">

</xml_diff>